<commit_message>
docs: finalize E1 hardware audit and reproducibility
</commit_message>
<xml_diff>
--- a/results/figures/e1/E1_grafici.xlsx
+++ b/results/figures/e1/E1_grafici.xlsx
@@ -2,13 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guida" sheetId="1" r:id="R434dd827293b4fb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grafici_E1" sheetId="2" r:id="R5ecb57061bd24fe2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validazione_v2" sheetId="3" r:id="R0480469028e24192"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_campagna" sheetId="4" r:id="Re199467239a34ecf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mac_test" sheetId="5" r:id="R490a1fbd5e6b4310"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mac_runs" sheetId="6" r:id="R6b7088581ab44795"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confronto_piattaforme" sheetId="7" r:id="Re02f89e23c8345a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guida" sheetId="1" r:id="R44a7dcd65b094bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grafici_E1" sheetId="2" r:id="R1382b36982794065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validazione_v2" sheetId="3" r:id="Ra081912cb4844c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test_campagna" sheetId="4" r:id="R10dcb8f1467b4c89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mac_test" sheetId="5" r:id="Rc0c5d95a75804376"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mac_runs" sheetId="6" r:id="Rbf0f27b96c674808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confronto_piattaforme" sheetId="7" r:id="Rfe1dccf93ffb4575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_hardware" sheetId="8" r:id="R45e32775143c42e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mac_val_standalone" sheetId="9" r:id="R35caccdd9099437e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,12 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0.000000"/>
     <x:numFmt numFmtId="201" formatCode="0.0000"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
+    <x:numFmt numFmtId="203" formatCode="0.000"/>
+    <x:numFmt numFmtId="204" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,8 +72,13 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF24444A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -101,6 +110,16 @@
         <x:fgColor rgb="FFE8F0F9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4F1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -109,7 +128,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -166,6 +185,25 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -284,6 +322,208 @@
         <c:axId val="48650112"/>
         <c:axId val="48672768"/>
       </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Media elapsed_sec per fit</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Audit_hardware'!$A$23:$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Audit_hardware'!$B$23:$B$24</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Mac mean elapsed_sec</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Audit_hardware'!$A$30:$A$33</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Audit_hardware'!$B$30:$B$33</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
       <c:catAx>
         <c:axId val="48650112"/>
         <c:scaling>
@@ -1472,7 +1712,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0986b5fdc3aa46af"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf7f88a47bfb74e08"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1502,7 +1742,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac5ae257c8cf4ee4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rece4971f2d17404b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1532,7 +1772,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb6d7a18ce51948be"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfba75caa9cdb45dc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1562,7 +1802,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d9a3e68786e4456"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R621dbc3bf9024ccd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1597,7 +1837,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc8a5bcbfba274d0f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R55dbb6bbd23a4aac"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1627,7 +1867,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3b97b6e6e8e4479f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re6586ddb61a14ead"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1657,7 +1897,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b89e9a503734e27"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9b917062aa0a49a7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1687,7 +1927,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf19e0299c30c4b1a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5032507e25d84848"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1717,7 +1957,72 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd61f5f846e524638"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8eb294cb8e614ea5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra822d5cbd0e943f9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad493b806b3942ee"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2506,7 +2811,7 @@
     <x:mergeCell ref="A11:M11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2290ccf9e97c43fe"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd642a226d4774bcf"/>
 </x:worksheet>
 </file>
 
@@ -3159,7 +3464,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c7b409beb7e4ee1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bb2d591460b42bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4373,7 +4678,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1461d6e2157548ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1353e0055f455c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29717,7 +30022,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>ATTENZIONE: commit Ubuntu test f5bf86b, Mac 59f556c. L’identità dei sorgenti del runner non è ancora verificata.</x:v>
+        <x:v>RUNNER: SHA-256 identico verificato; Fabrizio dichiara diff Git nullo sui file esecutivi. Rimane variabilità numerica TF.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -29735,6 +30040,1496 @@
     <x:mergeCell ref="A13:M13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34d9859b2e254829"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b87a90147a94a02"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="42" t="str">
+        <x:v>E1 · AUDIT HARDWARE E RIPRODUCIBILITÀ — 20 OTT 2026</x:v>
+      </x:c>
+      <x:c r="B1" s="42"/>
+      <x:c r="C1" s="42"/>
+      <x:c r="D1" s="42"/>
+      <x:c r="E1" s="42"/>
+      <x:c r="F1" s="42"/>
+      <x:c r="G1" s="42"/>
+      <x:c r="H1" s="42"/>
+      <x:c r="I1" s="42"/>
+      <x:c r="J1" s="42"/>
+      <x:c r="K1" s="42"/>
+      <x:c r="L1" s="42"/>
+      <x:c r="M1" s="42"/>
+      <x:c r="N1" s="42"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="43" t="str">
+        <x:v>Ubuntu 24.04 / VirtualBox x86_64 vs macOS / Apple M4 ARM64 · dati storici, nessun nuovo training</x:v>
+      </x:c>
+      <x:c r="B2" s="43"/>
+      <x:c r="C2" s="43"/>
+      <x:c r="D2" s="43"/>
+      <x:c r="E2" s="43"/>
+      <x:c r="F2" s="43"/>
+      <x:c r="G2" s="43"/>
+      <x:c r="H2" s="43"/>
+      <x:c r="I2" s="43"/>
+      <x:c r="J2" s="43"/>
+      <x:c r="K2" s="43"/>
+      <x:c r="L2" s="43"/>
+      <x:c r="M2" s="43"/>
+      <x:c r="N2" s="43"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="28"/>
+      <x:c r="B3" s="28"/>
+      <x:c r="C3" s="28"/>
+      <x:c r="D3" s="28"/>
+      <x:c r="E3" s="28"/>
+      <x:c r="F3" s="28"/>
+      <x:c r="G3" s="28"/>
+      <x:c r="H3" s="28"/>
+      <x:c r="I3" s="28"/>
+      <x:c r="J3" s="28"/>
+      <x:c r="K3" s="28"/>
+      <x:c r="L3" s="28"/>
+      <x:c r="M3" s="28"/>
+      <x:c r="N3" s="28"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="42" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="B4" s="42" t="str">
+        <x:v>AUROC Ubuntu</x:v>
+      </x:c>
+      <x:c r="C4" s="42" t="str">
+        <x:v>AUROC Mac</x:v>
+      </x:c>
+      <x:c r="D4" s="42" t="str">
+        <x:v>Delta Mac-Ubu</x:v>
+      </x:c>
+      <x:c r="E4" s="42" t="str">
+        <x:v>Mac standalone val AUROC</x:v>
+      </x:c>
+      <x:c r="F4" s="42" t="str">
+        <x:v>Mac val della campagna test AUROC</x:v>
+      </x:c>
+      <x:c r="G4" s="28"/>
+      <x:c r="H4" s="28"/>
+      <x:c r="I4" s="28"/>
+      <x:c r="J4" s="28"/>
+      <x:c r="K4" s="28"/>
+      <x:c r="L4" s="28"/>
+      <x:c r="M4" s="28"/>
+      <x:c r="N4" s="28"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="44" t="n">
+        <x:f>Confronto_piattaforme!B6</x:f>
+        <x:v>0.50015</x:v>
+      </x:c>
+      <x:c r="C5" s="44" t="n">
+        <x:f>Confronto_piattaforme!C6</x:f>
+        <x:v>0.50020875</x:v>
+      </x:c>
+      <x:c r="D5" s="44" t="n">
+        <x:f>C5-B5</x:f>
+        <x:v>0.000058749999999996305</x:v>
+      </x:c>
+      <x:c r="E5" s="44" t="n">
+        <x:v>0.50013375</x:v>
+      </x:c>
+      <x:c r="F5" s="44" t="n">
+        <x:f>Confronto_piattaforme!M6</x:f>
+        <x:v>0.5002537499999999</x:v>
+      </x:c>
+      <x:c r="G5" s="28"/>
+      <x:c r="H5" s="28"/>
+      <x:c r="I5" s="28"/>
+      <x:c r="J5" s="28"/>
+      <x:c r="K5" s="28"/>
+      <x:c r="L5" s="28"/>
+      <x:c r="M5" s="28"/>
+      <x:c r="N5" s="28"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="n">
+        <x:f>Confronto_piattaforme!B7</x:f>
+        <x:v>0.508232</x:v>
+      </x:c>
+      <x:c r="C6" s="44" t="n">
+        <x:f>Confronto_piattaforme!C7</x:f>
+        <x:v>0.5093875000000001</x:v>
+      </x:c>
+      <x:c r="D6" s="44" t="n">
+        <x:f>C6-B6</x:f>
+        <x:v>0.001155500000000087</x:v>
+      </x:c>
+      <x:c r="E6" s="44" t="n">
+        <x:v>0.49415000000000003</x:v>
+      </x:c>
+      <x:c r="F6" s="44" t="n">
+        <x:f>Confronto_piattaforme!M7</x:f>
+        <x:v>0.49582750000000003</x:v>
+      </x:c>
+      <x:c r="G6" s="28"/>
+      <x:c r="H6" s="28"/>
+      <x:c r="I6" s="28"/>
+      <x:c r="J6" s="28"/>
+      <x:c r="K6" s="28"/>
+      <x:c r="L6" s="28"/>
+      <x:c r="M6" s="28"/>
+      <x:c r="N6" s="28"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="28" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B7" s="44" t="n">
+        <x:f>Confronto_piattaforme!B8</x:f>
+        <x:v>0.501293</x:v>
+      </x:c>
+      <x:c r="C7" s="44" t="n">
+        <x:f>Confronto_piattaforme!C8</x:f>
+        <x:v>0.501425</x:v>
+      </x:c>
+      <x:c r="D7" s="44" t="n">
+        <x:f>C7-B7</x:f>
+        <x:v>0.000132000000000021</x:v>
+      </x:c>
+      <x:c r="E7" s="44" t="n">
+        <x:v>0.5039625</x:v>
+      </x:c>
+      <x:c r="F7" s="44" t="n">
+        <x:f>Confronto_piattaforme!M8</x:f>
+        <x:v>0.50266875</x:v>
+      </x:c>
+      <x:c r="G7" s="28"/>
+      <x:c r="H7" s="28"/>
+      <x:c r="I7" s="28"/>
+      <x:c r="J7" s="28"/>
+      <x:c r="K7" s="28"/>
+      <x:c r="L7" s="28"/>
+      <x:c r="M7" s="28"/>
+      <x:c r="N7" s="28"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="28" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B8" s="44" t="n">
+        <x:f>Confronto_piattaforme!B9</x:f>
+        <x:v>0.901863</x:v>
+      </x:c>
+      <x:c r="C8" s="44" t="n">
+        <x:f>Confronto_piattaforme!C9</x:f>
+        <x:v>0.9043775000000001</x:v>
+      </x:c>
+      <x:c r="D8" s="44" t="n">
+        <x:f>C8-B8</x:f>
+        <x:v>0.002514500000000086</x:v>
+      </x:c>
+      <x:c r="E8" s="44" t="n">
+        <x:v>0.8827</x:v>
+      </x:c>
+      <x:c r="F8" s="44" t="n">
+        <x:f>Confronto_piattaforme!M9</x:f>
+        <x:v>0.8830275000000001</x:v>
+      </x:c>
+      <x:c r="G8" s="28"/>
+      <x:c r="H8" s="28"/>
+      <x:c r="I8" s="28"/>
+      <x:c r="J8" s="28"/>
+      <x:c r="K8" s="28"/>
+      <x:c r="L8" s="28"/>
+      <x:c r="M8" s="28"/>
+      <x:c r="N8" s="28"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="28"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
+      <x:c r="H9" s="28"/>
+      <x:c r="I9" s="28"/>
+      <x:c r="J9" s="28"/>
+      <x:c r="K9" s="28"/>
+      <x:c r="L9" s="28"/>
+      <x:c r="M9" s="28"/>
+      <x:c r="N9" s="28"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="28"/>
+      <x:c r="B10" s="28"/>
+      <x:c r="C10" s="28"/>
+      <x:c r="D10" s="28"/>
+      <x:c r="E10" s="28"/>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28"/>
+      <x:c r="H10" s="28"/>
+      <x:c r="I10" s="28"/>
+      <x:c r="J10" s="28"/>
+      <x:c r="K10" s="28"/>
+      <x:c r="L10" s="28"/>
+      <x:c r="M10" s="28"/>
+      <x:c r="N10" s="28"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="42" t="str">
+        <x:v>CONTROLLO DELLA PROVENIENZA — livelli diversi di verifica</x:v>
+      </x:c>
+      <x:c r="B11" s="42"/>
+      <x:c r="C11" s="42"/>
+      <x:c r="D11" s="42"/>
+      <x:c r="E11" s="42"/>
+      <x:c r="F11" s="42"/>
+      <x:c r="G11" s="42"/>
+      <x:c r="H11" s="42"/>
+      <x:c r="I11" s="42"/>
+      <x:c r="J11" s="42"/>
+      <x:c r="K11" s="42"/>
+      <x:c r="L11" s="42"/>
+      <x:c r="M11" s="42"/>
+      <x:c r="N11" s="42"/>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="28" t="str">
+        <x:v>Codice runner</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="str">
+        <x:v>SHA-256 locale verificato: a75aa3d844bb695a6d6155fe808394025b04c480d74d1e1b856eec5ca6f9c037</x:v>
+      </x:c>
+      <x:c r="C12" s="28"/>
+      <x:c r="D12" s="28"/>
+      <x:c r="E12" s="28"/>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28"/>
+      <x:c r="H12" s="28"/>
+      <x:c r="I12" s="28"/>
+      <x:c r="J12" s="28"/>
+      <x:c r="K12" s="28"/>
+      <x:c r="L12" s="28"/>
+      <x:c r="M12" s="28"/>
+      <x:c r="N12" s="28"/>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="28" t="str">
+        <x:v>Diff Git f5bf86b → 59f556c</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="str">
+        <x:v>Fabrizio comunica diff vuoto sui file esecutivi; output diff non incluso nello ZIP</x:v>
+      </x:c>
+      <x:c r="C13" s="28"/>
+      <x:c r="D13" s="28"/>
+      <x:c r="E13" s="28"/>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28"/>
+      <x:c r="H13" s="28"/>
+      <x:c r="I13" s="28"/>
+      <x:c r="J13" s="28"/>
+      <x:c r="K13" s="28"/>
+      <x:c r="L13" s="28"/>
+      <x:c r="M13" s="28"/>
+      <x:c r="N13" s="28"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="28" t="str">
+        <x:v>Pesi e split</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="str">
+        <x:v>SHA-256 identici nei run_config originali, verificato</x:v>
+      </x:c>
+      <x:c r="C14" s="28"/>
+      <x:c r="D14" s="28"/>
+      <x:c r="E14" s="28"/>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28"/>
+      <x:c r="H14" s="28"/>
+      <x:c r="I14" s="28"/>
+      <x:c r="J14" s="28"/>
+      <x:c r="K14" s="28"/>
+      <x:c r="L14" s="28"/>
+      <x:c r="M14" s="28"/>
+      <x:c r="N14" s="28"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="28" t="str">
+        <x:v>Payload repeat=0 / X=23</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="str">
+        <x:v>403/403 SHA-256 rigenerati con PCG64 e seed per identità: OK</x:v>
+      </x:c>
+      <x:c r="C15" s="28"/>
+      <x:c r="D15" s="28"/>
+      <x:c r="E15" s="28"/>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28"/>
+      <x:c r="H15" s="28"/>
+      <x:c r="I15" s="28"/>
+      <x:c r="J15" s="28"/>
+      <x:c r="K15" s="28"/>
+      <x:c r="L15" s="28"/>
+      <x:c r="M15" s="28"/>
+      <x:c r="N15" s="28"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="28" t="str">
+        <x:v>Mac test</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="str">
+        <x:v>320 righe metriche: 40 fit unici con 2 stage × 2 metodi × 2 politiche</x:v>
+      </x:c>
+      <x:c r="C16" s="28"/>
+      <x:c r="D16" s="28"/>
+      <x:c r="E16" s="28"/>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28"/>
+      <x:c r="H16" s="28"/>
+      <x:c r="I16" s="28"/>
+      <x:c r="J16" s="28"/>
+      <x:c r="K16" s="28"/>
+      <x:c r="L16" s="28"/>
+      <x:c r="M16" s="28"/>
+      <x:c r="N16" s="28"/>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="28" t="str">
+        <x:v>Mac validation separata</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="str">
+        <x:v>16 righe aggregate: 40 fit dichiarati; non incluso CSV per-run della campagna separata</x:v>
+      </x:c>
+      <x:c r="C17" s="28"/>
+      <x:c r="D17" s="28"/>
+      <x:c r="E17" s="28"/>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28"/>
+      <x:c r="H17" s="28"/>
+      <x:c r="I17" s="28"/>
+      <x:c r="J17" s="28"/>
+      <x:c r="K17" s="28"/>
+      <x:c r="L17" s="28"/>
+      <x:c r="M17" s="28"/>
+      <x:c r="N17" s="28"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="28" t="str">
+        <x:v>Precisione hardware</x:v>
+      </x:c>
+      <x:c r="B18" s="28" t="str">
+        <x:v>Confronto di ambienti, non causalità attribuibile al solo chip M4</x:v>
+      </x:c>
+      <x:c r="C18" s="28"/>
+      <x:c r="D18" s="28"/>
+      <x:c r="E18" s="28"/>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28"/>
+      <x:c r="H18" s="28"/>
+      <x:c r="I18" s="28"/>
+      <x:c r="J18" s="28"/>
+      <x:c r="K18" s="28"/>
+      <x:c r="L18" s="28"/>
+      <x:c r="M18" s="28"/>
+      <x:c r="N18" s="28"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="28" t="str">
+        <x:v>Memoria/tempo end-to-end</x:v>
+      </x:c>
+      <x:c r="B19" s="28" t="str">
+        <x:v>NON misurati in modo comparabile: benchmark opzionale</x:v>
+      </x:c>
+      <x:c r="C19" s="28"/>
+      <x:c r="D19" s="28"/>
+      <x:c r="E19" s="28"/>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28"/>
+      <x:c r="H19" s="28"/>
+      <x:c r="I19" s="28"/>
+      <x:c r="J19" s="28"/>
+      <x:c r="K19" s="28"/>
+      <x:c r="L19" s="28"/>
+      <x:c r="M19" s="28"/>
+      <x:c r="N19" s="28"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="28"/>
+      <x:c r="B20" s="28"/>
+      <x:c r="C20" s="28"/>
+      <x:c r="D20" s="28"/>
+      <x:c r="E20" s="28"/>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28"/>
+      <x:c r="H20" s="28"/>
+      <x:c r="I20" s="28"/>
+      <x:c r="J20" s="28"/>
+      <x:c r="K20" s="28"/>
+      <x:c r="L20" s="28"/>
+      <x:c r="M20" s="28"/>
+      <x:c r="N20" s="28"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="28"/>
+      <x:c r="B21" s="28"/>
+      <x:c r="C21" s="28"/>
+      <x:c r="D21" s="28"/>
+      <x:c r="E21" s="28"/>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28"/>
+      <x:c r="H21" s="28"/>
+      <x:c r="I21" s="28"/>
+      <x:c r="J21" s="28"/>
+      <x:c r="K21" s="28"/>
+      <x:c r="L21" s="28"/>
+      <x:c r="M21" s="28"/>
+      <x:c r="N21" s="28"/>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="42" t="str">
+        <x:v>Ambiente</x:v>
+      </x:c>
+      <x:c r="B22" s="42" t="str">
+        <x:v>Media elapsed_sec per fit</x:v>
+      </x:c>
+      <x:c r="C22" s="42" t="str">
+        <x:v>Fonte</x:v>
+      </x:c>
+      <x:c r="D22" s="28"/>
+      <x:c r="E22" s="28"/>
+      <x:c r="F22" s="28"/>
+      <x:c r="G22" s="28"/>
+      <x:c r="H22" s="28"/>
+      <x:c r="I22" s="28"/>
+      <x:c r="J22" s="28"/>
+      <x:c r="K22" s="28"/>
+      <x:c r="L22" s="28"/>
+      <x:c r="M22" s="28"/>
+      <x:c r="N22" s="28"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="28" t="str">
+        <x:v>Ubuntu VirtualBox</x:v>
+      </x:c>
+      <x:c r="B23" s="45" t="n">
+        <x:v>217.124</x:v>
+      </x:c>
+      <x:c r="C23" s="28" t="str">
+        <x:v>Audit locale Riccardo, 40 fit</x:v>
+      </x:c>
+      <x:c r="D23" s="28"/>
+      <x:c r="E23" s="28"/>
+      <x:c r="F23" s="28"/>
+      <x:c r="G23" s="28"/>
+      <x:c r="H23" s="28"/>
+      <x:c r="I23" s="28"/>
+      <x:c r="J23" s="28"/>
+      <x:c r="K23" s="28"/>
+      <x:c r="L23" s="28"/>
+      <x:c r="M23" s="28"/>
+      <x:c r="N23" s="28"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="28" t="str">
+        <x:v>Mac M4 CPU</x:v>
+      </x:c>
+      <x:c r="B24" s="45" t="n">
+        <x:v>104.412</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="str">
+        <x:v>CSV Mac originale, 40 fit</x:v>
+      </x:c>
+      <x:c r="D24" s="28"/>
+      <x:c r="E24" s="28"/>
+      <x:c r="F24" s="28"/>
+      <x:c r="G24" s="28"/>
+      <x:c r="H24" s="28"/>
+      <x:c r="I24" s="28"/>
+      <x:c r="J24" s="28"/>
+      <x:c r="K24" s="28"/>
+      <x:c r="L24" s="28"/>
+      <x:c r="M24" s="28"/>
+      <x:c r="N24" s="28"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="28"/>
+      <x:c r="B25" s="45"/>
+      <x:c r="C25" s="28"/>
+      <x:c r="D25" s="28"/>
+      <x:c r="E25" s="28"/>
+      <x:c r="F25" s="28"/>
+      <x:c r="G25" s="28"/>
+      <x:c r="H25" s="28"/>
+      <x:c r="I25" s="28"/>
+      <x:c r="J25" s="28"/>
+      <x:c r="K25" s="28"/>
+      <x:c r="L25" s="28"/>
+      <x:c r="M25" s="28"/>
+      <x:c r="N25" s="28"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="28" t="str">
+        <x:v>Rapporto medie Ubuntu/Mac</x:v>
+      </x:c>
+      <x:c r="B26" s="45" t="n">
+        <x:f>B23/B24</x:f>
+        <x:v>2.079492778607823</x:v>
+      </x:c>
+      <x:c r="C26" s="28"/>
+      <x:c r="D26" s="28"/>
+      <x:c r="E26" s="28"/>
+      <x:c r="F26" s="28"/>
+      <x:c r="G26" s="28"/>
+      <x:c r="H26" s="28"/>
+      <x:c r="I26" s="28"/>
+      <x:c r="J26" s="28"/>
+      <x:c r="K26" s="28"/>
+      <x:c r="L26" s="28"/>
+      <x:c r="M26" s="28"/>
+      <x:c r="N26" s="28"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="28"/>
+      <x:c r="B27" s="28"/>
+      <x:c r="C27" s="28"/>
+      <x:c r="D27" s="28"/>
+      <x:c r="E27" s="28"/>
+      <x:c r="F27" s="28"/>
+      <x:c r="G27" s="28"/>
+      <x:c r="H27" s="28"/>
+      <x:c r="I27" s="28"/>
+      <x:c r="J27" s="28"/>
+      <x:c r="K27" s="28"/>
+      <x:c r="L27" s="28"/>
+      <x:c r="M27" s="28"/>
+      <x:c r="N27" s="28"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="28"/>
+      <x:c r="B28" s="28"/>
+      <x:c r="C28" s="28"/>
+      <x:c r="D28" s="28"/>
+      <x:c r="E28" s="28"/>
+      <x:c r="F28" s="28"/>
+      <x:c r="G28" s="28"/>
+      <x:c r="H28" s="28"/>
+      <x:c r="I28" s="28"/>
+      <x:c r="J28" s="28"/>
+      <x:c r="K28" s="28"/>
+      <x:c r="L28" s="28"/>
+      <x:c r="M28" s="28"/>
+      <x:c r="N28" s="28"/>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="42" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="B29" s="42" t="str">
+        <x:v>Mac mean elapsed_sec</x:v>
+      </x:c>
+      <x:c r="C29" s="42" t="str">
+        <x:v>Mac SD elapsed_sec</x:v>
+      </x:c>
+      <x:c r="D29" s="28"/>
+      <x:c r="E29" s="28"/>
+      <x:c r="F29" s="28"/>
+      <x:c r="G29" s="28"/>
+      <x:c r="H29" s="28"/>
+      <x:c r="I29" s="28"/>
+      <x:c r="J29" s="28"/>
+      <x:c r="K29" s="28"/>
+      <x:c r="L29" s="28"/>
+      <x:c r="M29" s="28"/>
+      <x:c r="N29" s="28"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B30" s="46" t="n">
+        <x:v>102.757</x:v>
+      </x:c>
+      <x:c r="C30" s="46" t="n">
+        <x:v>5.966031716681068</x:v>
+      </x:c>
+      <x:c r="D30" s="28"/>
+      <x:c r="E30" s="28"/>
+      <x:c r="F30" s="28"/>
+      <x:c r="G30" s="28"/>
+      <x:c r="H30" s="28"/>
+      <x:c r="I30" s="28"/>
+      <x:c r="J30" s="28"/>
+      <x:c r="K30" s="28"/>
+      <x:c r="L30" s="28"/>
+      <x:c r="M30" s="28"/>
+      <x:c r="N30" s="28"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="28" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B31" s="46" t="n">
+        <x:v>104.223</x:v>
+      </x:c>
+      <x:c r="C31" s="46" t="n">
+        <x:v>2.3641961283559634</x:v>
+      </x:c>
+      <x:c r="D31" s="28"/>
+      <x:c r="E31" s="28"/>
+      <x:c r="F31" s="28"/>
+      <x:c r="G31" s="28"/>
+      <x:c r="H31" s="28"/>
+      <x:c r="I31" s="28"/>
+      <x:c r="J31" s="28"/>
+      <x:c r="K31" s="28"/>
+      <x:c r="L31" s="28"/>
+      <x:c r="M31" s="28"/>
+      <x:c r="N31" s="28"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="28" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B32" s="46" t="n">
+        <x:v>105.124</x:v>
+      </x:c>
+      <x:c r="C32" s="46" t="n">
+        <x:v>1.7309483592014605</x:v>
+      </x:c>
+      <x:c r="D32" s="28"/>
+      <x:c r="E32" s="28"/>
+      <x:c r="F32" s="28"/>
+      <x:c r="G32" s="28"/>
+      <x:c r="H32" s="28"/>
+      <x:c r="I32" s="28"/>
+      <x:c r="J32" s="28"/>
+      <x:c r="K32" s="28"/>
+      <x:c r="L32" s="28"/>
+      <x:c r="M32" s="28"/>
+      <x:c r="N32" s="28"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="28" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B33" s="46" t="n">
+        <x:v>105.544</x:v>
+      </x:c>
+      <x:c r="C33" s="46" t="n">
+        <x:v>1.4096508629996132</x:v>
+      </x:c>
+      <x:c r="D33" s="28"/>
+      <x:c r="E33" s="28"/>
+      <x:c r="F33" s="28"/>
+      <x:c r="G33" s="28"/>
+      <x:c r="H33" s="28"/>
+      <x:c r="I33" s="28"/>
+      <x:c r="J33" s="28"/>
+      <x:c r="K33" s="28"/>
+      <x:c r="L33" s="28"/>
+      <x:c r="M33" s="28"/>
+      <x:c r="N33" s="28"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="28"/>
+      <x:c r="B34" s="28"/>
+      <x:c r="C34" s="28"/>
+      <x:c r="D34" s="28"/>
+      <x:c r="E34" s="28"/>
+      <x:c r="F34" s="28"/>
+      <x:c r="G34" s="28"/>
+      <x:c r="H34" s="28"/>
+      <x:c r="I34" s="28"/>
+      <x:c r="J34" s="28"/>
+      <x:c r="K34" s="28"/>
+      <x:c r="L34" s="28"/>
+      <x:c r="M34" s="28"/>
+      <x:c r="N34" s="28"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="28"/>
+      <x:c r="B35" s="28"/>
+      <x:c r="C35" s="28"/>
+      <x:c r="D35" s="28"/>
+      <x:c r="E35" s="28"/>
+      <x:c r="F35" s="28"/>
+      <x:c r="G35" s="28"/>
+      <x:c r="H35" s="28"/>
+      <x:c r="I35" s="28"/>
+      <x:c r="J35" s="28"/>
+      <x:c r="K35" s="28"/>
+      <x:c r="L35" s="28"/>
+      <x:c r="M35" s="28"/>
+      <x:c r="N35" s="28"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="28" t="str">
+        <x:v>Nota: elapsed_sec esclude avvio processo e alcune fasi di preparazione; NON è durata end-to-end.</x:v>
+      </x:c>
+      <x:c r="B36" s="28"/>
+      <x:c r="C36" s="28"/>
+      <x:c r="D36" s="28"/>
+      <x:c r="E36" s="28"/>
+      <x:c r="F36" s="28"/>
+      <x:c r="G36" s="28"/>
+      <x:c r="H36" s="28"/>
+      <x:c r="I36" s="28"/>
+      <x:c r="J36" s="28"/>
+      <x:c r="K36" s="28"/>
+      <x:c r="L36" s="28"/>
+      <x:c r="M36" s="28"/>
+      <x:c r="N36" s="28"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="28"/>
+      <x:c r="B37" s="28"/>
+      <x:c r="C37" s="28"/>
+      <x:c r="D37" s="28"/>
+      <x:c r="E37" s="28"/>
+      <x:c r="F37" s="28"/>
+      <x:c r="G37" s="28"/>
+      <x:c r="H37" s="28"/>
+      <x:c r="I37" s="28"/>
+      <x:c r="J37" s="28"/>
+      <x:c r="K37" s="28"/>
+      <x:c r="L37" s="28"/>
+      <x:c r="M37" s="28"/>
+      <x:c r="N37" s="28"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="28"/>
+      <x:c r="B38" s="28"/>
+      <x:c r="C38" s="28"/>
+      <x:c r="D38" s="28"/>
+      <x:c r="E38" s="28"/>
+      <x:c r="F38" s="28"/>
+      <x:c r="G38" s="28"/>
+      <x:c r="H38" s="28"/>
+      <x:c r="I38" s="28"/>
+      <x:c r="J38" s="28"/>
+      <x:c r="K38" s="28"/>
+      <x:c r="L38" s="28"/>
+      <x:c r="M38" s="28"/>
+      <x:c r="N38" s="28"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="28"/>
+      <x:c r="B39" s="28"/>
+      <x:c r="C39" s="28"/>
+      <x:c r="D39" s="28"/>
+      <x:c r="E39" s="28"/>
+      <x:c r="F39" s="28"/>
+      <x:c r="G39" s="28"/>
+      <x:c r="H39" s="28"/>
+      <x:c r="I39" s="28"/>
+      <x:c r="J39" s="28"/>
+      <x:c r="K39" s="28"/>
+      <x:c r="L39" s="28"/>
+      <x:c r="M39" s="28"/>
+      <x:c r="N39" s="28"/>
+    </x:row>
+    <x:row r="56" ht="27" customHeight="1">
+      <x:c r="A56" t="str">
+        <x:v>Nota: differenze per 10 fit appaiati ottenibili dai file locali di Riccardo con scripts/audit_e1_platforms.py.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
+    <x:mergeCell ref="A11:N11"/>
+    <x:mergeCell ref="A36:N36"/>
+    <x:mergeCell ref="B12:F12"/>
+    <x:mergeCell ref="B13:F13"/>
+    <x:mergeCell ref="B14:F14"/>
+    <x:mergeCell ref="B15:F15"/>
+    <x:mergeCell ref="B16:F16"/>
+    <x:mergeCell ref="B17:F17"/>
+    <x:mergeCell ref="B18:F18"/>
+    <x:mergeCell ref="B19:F19"/>
+    <x:mergeCell ref="A56:N56"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c2fea60fb0345ec"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="39" t="str">
+        <x:v>MAC M4 — VALIDATION STAND-ALONE (40 FIT, SUMMARY DI FABRIZIO)</x:v>
+      </x:c>
+      <x:c r="B1" s="39"/>
+      <x:c r="C1" s="39"/>
+      <x:c r="D1" s="39"/>
+      <x:c r="E1" s="39"/>
+      <x:c r="F1" s="39"/>
+      <x:c r="G1" s="39"/>
+      <x:c r="H1" s="39"/>
+      <x:c r="I1" s="39"/>
+      <x:c r="J1" s="39"/>
+      <x:c r="K1" s="39"/>
+    </x:row>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="41" t="str">
+        <x:v>Non confondere con la validation ri-calcolata durante la campagna test.</x:v>
+      </x:c>
+      <x:c r="B2" s="41"/>
+      <x:c r="C2" s="41"/>
+      <x:c r="D2" s="41"/>
+      <x:c r="E2" s="41"/>
+      <x:c r="F2" s="41"/>
+      <x:c r="G2" s="41"/>
+      <x:c r="H2" s="41"/>
+      <x:c r="I2" s="41"/>
+      <x:c r="J2" s="41"/>
+      <x:c r="K2" s="41"/>
+    </x:row>
+    <x:row r="4" ht="23" customHeight="1">
+      <x:c r="A4" s="39" t="str">
+        <x:v>stage</x:v>
+      </x:c>
+      <x:c r="B4" s="39" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C4" s="39" t="str">
+        <x:v>method</x:v>
+      </x:c>
+      <x:c r="D4" s="39" t="str">
+        <x:v>policy</x:v>
+      </x:c>
+      <x:c r="E4" s="39" t="str">
+        <x:v>n_runs</x:v>
+      </x:c>
+      <x:c r="F4" s="39" t="str">
+        <x:v>accuracy_mean</x:v>
+      </x:c>
+      <x:c r="G4" s="39" t="str">
+        <x:v>accuracy_std</x:v>
+      </x:c>
+      <x:c r="H4" s="39" t="str">
+        <x:v>auroc_mean</x:v>
+      </x:c>
+      <x:c r="I4" s="39" t="str">
+        <x:v>auprc_mean</x:v>
+      </x:c>
+      <x:c r="J4" s="39" t="str">
+        <x:v>f1_mean</x:v>
+      </x:c>
+      <x:c r="K4" s="39" t="str">
+        <x:v>fpr_mean</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="16" t="n">
+        <x:v>0.49974999999999997</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="n">
+        <x:v>0.0014191155304938588</x:v>
+      </x:c>
+      <x:c r="H5" s="16" t="n">
+        <x:v>0.50013375</x:v>
+      </x:c>
+      <x:c r="I5" s="16" t="n">
+        <x:v>0.5045302615999082</x:v>
+      </x:c>
+      <x:c r="J5" s="16" t="n">
+        <x:v>0.47171177344603593</x:v>
+      </x:c>
+      <x:c r="K5" s="16" t="n">
+        <x:v>0.49450000000000005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="16" t="n">
+        <x:v>0.5085</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="n">
+        <x:v>0.0017480147469502933</x:v>
+      </x:c>
+      <x:c r="H6" s="16" t="n">
+        <x:v>0.50013375</x:v>
+      </x:c>
+      <x:c r="I6" s="16" t="n">
+        <x:v>0.5045302615999082</x:v>
+      </x:c>
+      <x:c r="J6" s="16" t="n">
+        <x:v>0.455841371964614</x:v>
+      </x:c>
+      <x:c r="K6" s="16" t="n">
+        <x:v>0.4505</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="16" t="n">
+        <x:v>0.5005</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="n">
+        <x:v>0.0022973414586816947</x:v>
+      </x:c>
+      <x:c r="H7" s="16" t="n">
+        <x:v>0.5006412499999999</x:v>
+      </x:c>
+      <x:c r="I7" s="16" t="n">
+        <x:v>0.5053104581554917</x:v>
+      </x:c>
+      <x:c r="J7" s="16" t="n">
+        <x:v>0.5188732465183853</x:v>
+      </x:c>
+      <x:c r="K7" s="16" t="n">
+        <x:v>0.5660000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="n">
+        <x:v>0.5085</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="n">
+        <x:v>0.001290994448735837</x:v>
+      </x:c>
+      <x:c r="H8" s="16" t="n">
+        <x:v>0.5006412499999999</x:v>
+      </x:c>
+      <x:c r="I8" s="16" t="n">
+        <x:v>0.5053104581554917</x:v>
+      </x:c>
+      <x:c r="J8" s="16" t="n">
+        <x:v>0.47381468481010625</x:v>
+      </x:c>
+      <x:c r="K8" s="16" t="n">
+        <x:v>0.4885</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F9" s="16" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="n">
+        <x:v>0.01649915822768608</x:v>
+      </x:c>
+      <x:c r="H9" s="16" t="n">
+        <x:v>0.49415000000000003</x:v>
+      </x:c>
+      <x:c r="I9" s="16" t="n">
+        <x:v>0.5010644778484645</x:v>
+      </x:c>
+      <x:c r="J9" s="16" t="n">
+        <x:v>0.4903008997150649</x:v>
+      </x:c>
+      <x:c r="K9" s="16" t="n">
+        <x:v>0.533</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F10" s="16" t="n">
+        <x:v>0.52475</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="n">
+        <x:v>0.011513880511992668</x:v>
+      </x:c>
+      <x:c r="H10" s="16" t="n">
+        <x:v>0.49415000000000003</x:v>
+      </x:c>
+      <x:c r="I10" s="16" t="n">
+        <x:v>0.5010644778484645</x:v>
+      </x:c>
+      <x:c r="J10" s="16" t="n">
+        <x:v>0.42965139309676365</x:v>
+      </x:c>
+      <x:c r="K10" s="16" t="n">
+        <x:v>0.4205</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="16" t="n">
+        <x:v>0.50225</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="n">
+        <x:v>0.02373025495016857</x:v>
+      </x:c>
+      <x:c r="H11" s="16" t="n">
+        <x:v>0.499645</x:v>
+      </x:c>
+      <x:c r="I11" s="16" t="n">
+        <x:v>0.5021262217635386</x:v>
+      </x:c>
+      <x:c r="J11" s="16" t="n">
+        <x:v>0.49476881942122775</x:v>
+      </x:c>
+      <x:c r="K11" s="16" t="n">
+        <x:v>0.5469999999999999</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F12" s="16" t="n">
+        <x:v>0.53025</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="n">
+        <x:v>0.01626388295853388</x:v>
+      </x:c>
+      <x:c r="H12" s="16" t="n">
+        <x:v>0.499645</x:v>
+      </x:c>
+      <x:c r="I12" s="16" t="n">
+        <x:v>0.5021262217635386</x:v>
+      </x:c>
+      <x:c r="J12" s="16" t="n">
+        <x:v>0.5437944320660918</x:v>
+      </x:c>
+      <x:c r="K12" s="16" t="n">
+        <x:v>0.5650000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F13" s="16" t="n">
+        <x:v>0.4995</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="n">
+        <x:v>0.02365257796614238</x:v>
+      </x:c>
+      <x:c r="H13" s="16" t="n">
+        <x:v>0.5039625</x:v>
+      </x:c>
+      <x:c r="I13" s="16" t="n">
+        <x:v>0.5186567562577401</x:v>
+      </x:c>
+      <x:c r="J13" s="16" t="n">
+        <x:v>0.45967428378038794</x:v>
+      </x:c>
+      <x:c r="K13" s="16" t="n">
+        <x:v>0.4445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F14" s="16" t="n">
+        <x:v>0.53575</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="n">
+        <x:v>0.01086853255964206</x:v>
+      </x:c>
+      <x:c r="H14" s="16" t="n">
+        <x:v>0.5039625</x:v>
+      </x:c>
+      <x:c r="I14" s="16" t="n">
+        <x:v>0.5186567562577401</x:v>
+      </x:c>
+      <x:c r="J14" s="16" t="n">
+        <x:v>0.4115469803892702</x:v>
+      </x:c>
+      <x:c r="K14" s="16" t="n">
+        <x:v>0.3235</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="n">
+        <x:v>0.5125</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="n">
+        <x:v>0.02058181505871413</x:v>
+      </x:c>
+      <x:c r="H15" s="16" t="n">
+        <x:v>0.5076612500000001</x:v>
+      </x:c>
+      <x:c r="I15" s="16" t="n">
+        <x:v>0.5086367222307453</x:v>
+      </x:c>
+      <x:c r="J15" s="16" t="n">
+        <x:v>0.5156389058377085</x:v>
+      </x:c>
+      <x:c r="K15" s="16" t="n">
+        <x:v>0.5285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F16" s="16" t="n">
+        <x:v>0.5349999999999999</x:v>
+      </x:c>
+      <x:c r="G16" s="16" t="n">
+        <x:v>0.017320508075688825</x:v>
+      </x:c>
+      <x:c r="H16" s="16" t="n">
+        <x:v>0.5076612500000001</x:v>
+      </x:c>
+      <x:c r="I16" s="16" t="n">
+        <x:v>0.5086367222307453</x:v>
+      </x:c>
+      <x:c r="J16" s="16" t="n">
+        <x:v>0.5054145693632323</x:v>
+      </x:c>
+      <x:c r="K16" s="16" t="n">
+        <x:v>0.4655</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B17" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F17" s="16" t="n">
+        <x:v>0.78625</x:v>
+      </x:c>
+      <x:c r="G17" s="16" t="n">
+        <x:v>0.07366638386069396</x:v>
+      </x:c>
+      <x:c r="H17" s="16" t="n">
+        <x:v>0.8827</x:v>
+      </x:c>
+      <x:c r="I17" s="16" t="n">
+        <x:v>0.879341885861413</x:v>
+      </x:c>
+      <x:c r="J17" s="16" t="n">
+        <x:v>0.777444175854068</x:v>
+      </x:c>
+      <x:c r="K17" s="16" t="n">
+        <x:v>0.19849999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>centroid</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E18" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F18" s="16" t="n">
+        <x:v>0.8192499999999999</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="n">
+        <x:v>0.06664635107124099</x:v>
+      </x:c>
+      <x:c r="H18" s="16" t="n">
+        <x:v>0.8827</x:v>
+      </x:c>
+      <x:c r="I18" s="16" t="n">
+        <x:v>0.879341885861413</x:v>
+      </x:c>
+      <x:c r="J18" s="16" t="n">
+        <x:v>0.8164102191503819</x:v>
+      </x:c>
+      <x:c r="K18" s="16" t="n">
+        <x:v>0.1775</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B19" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>original_zero</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F19" s="16" t="n">
+        <x:v>0.7125</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="n">
+        <x:v>0.06999007866198685</x:v>
+      </x:c>
+      <x:c r="H19" s="16" t="n">
+        <x:v>0.80254625</x:v>
+      </x:c>
+      <x:c r="I19" s="16" t="n">
+        <x:v>0.798394093356284</x:v>
+      </x:c>
+      <x:c r="J19" s="16" t="n">
+        <x:v>0.7254395417415539</x:v>
+      </x:c>
+      <x:c r="K19" s="16" t="n">
+        <x:v>0.3315</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>validation</x:v>
+      </x:c>
+      <x:c r="B20" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>nn</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>val_youden</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F20" s="16" t="n">
+        <x:v>0.74075</x:v>
+      </x:c>
+      <x:c r="G20" s="16" t="n">
+        <x:v>0.05816702483175308</x:v>
+      </x:c>
+      <x:c r="H20" s="16" t="n">
+        <x:v>0.80254625</x:v>
+      </x:c>
+      <x:c r="I20" s="16" t="n">
+        <x:v>0.798394093356284</x:v>
+      </x:c>
+      <x:c r="J20" s="16" t="n">
+        <x:v>0.7457086803902268</x:v>
+      </x:c>
+      <x:c r="K20" s="16" t="n">
+        <x:v>0.2805</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>